<commit_message>
🎉 add: TickTimer 초안 추가
</commit_message>
<xml_diff>
--- a/Server/Common/GameDatasheet/Original_Monster.xlsx
+++ b/Server/Common/GameDatasheet/Original_Monster.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zmwps\Desktop\Project_MMORPG\Server\Common\GameDatasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED19BA6-8190-44C6-8A41-C0515D7B9B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45BC756-4F2C-420E-BFFD-E48E38C4BB5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5520" yWindow="1656" windowWidth="24828" windowHeight="12204" xr2:uid="{1E70E408-E624-4B81-99D5-889082593FF6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{1E70E408-E624-4B81-99D5-889082593FF6}"/>
   </bookViews>
   <sheets>
     <sheet name="몬스터(5000~5999)" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,82 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>윤형석</author>
+  </authors>
+  <commentList>
+    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{C371950D-C514-4F32-9E11-F3BC3AC117EC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="돋움"/>
+            <family val="3"/>
+            <charset val="129"/>
+          </rPr>
+          <t>윤형석</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="돋움"/>
+            <family val="3"/>
+            <charset val="129"/>
+          </rPr>
+          <t>공격</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="돋움"/>
+            <family val="3"/>
+            <charset val="129"/>
+          </rPr>
+          <t>사거리</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
   <si>
     <t>monster_name</t>
   </si>
@@ -222,6 +296,10 @@
   </si>
   <si>
     <t>"/Game/Blueprints/Creatures/Monster/SuperMonster/BP_Expert_SuperMinion.BP_Expert_SuperMinion_C"</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>attack_attack_range</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -229,7 +307,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -244,6 +322,34 @@
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="2">
@@ -585,14 +691,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{424A49E2-B413-473B-95D1-65DE3060862F}">
-  <dimension ref="A1:M11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{424A49E2-B413-473B-95D1-65DE3060862F}">
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -624,16 +730,19 @@
         <v>5</v>
       </c>
       <c r="K1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>7</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -671,10 +780,13 @@
         <v>20</v>
       </c>
       <c r="M2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>5000</v>
       </c>
@@ -703,19 +815,23 @@
         <v>1</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K3">
-        <v>3</v>
+        <f>J3-50</f>
+        <v>50</v>
       </c>
       <c r="L3">
-        <v>5</v>
-      </c>
-      <c r="M3" t="s">
+        <v>800</v>
+      </c>
+      <c r="M3">
+        <v>1500</v>
+      </c>
+      <c r="N3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>5001</v>
       </c>
@@ -744,19 +860,23 @@
         <v>1</v>
       </c>
       <c r="J4">
-        <v>5</v>
+        <v>800</v>
       </c>
       <c r="K4">
-        <v>3</v>
+        <f>J4-100</f>
+        <v>700</v>
       </c>
       <c r="L4">
-        <v>5</v>
-      </c>
-      <c r="M4" t="s">
+        <v>800</v>
+      </c>
+      <c r="M4">
+        <v>1500</v>
+      </c>
+      <c r="N4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>5002</v>
       </c>
@@ -785,19 +905,23 @@
         <v>1</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <f t="shared" ref="K4:K11" si="0">J5-50</f>
+        <v>50</v>
       </c>
       <c r="L5">
-        <v>5</v>
-      </c>
-      <c r="M5" t="s">
+        <v>800</v>
+      </c>
+      <c r="M5">
+        <v>1500</v>
+      </c>
+      <c r="N5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>5003</v>
       </c>
@@ -826,19 +950,23 @@
         <v>1</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K6">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6" t="s">
+        <v>800</v>
+      </c>
+      <c r="M6">
+        <v>1500</v>
+      </c>
+      <c r="N6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>5004</v>
       </c>
@@ -867,19 +995,23 @@
         <v>1</v>
       </c>
       <c r="J7">
-        <v>5</v>
+        <v>800</v>
       </c>
       <c r="K7">
-        <v>3</v>
+        <f>J7-100</f>
+        <v>700</v>
       </c>
       <c r="L7">
-        <v>5</v>
-      </c>
-      <c r="M7" t="s">
+        <v>800</v>
+      </c>
+      <c r="M7">
+        <v>1500</v>
+      </c>
+      <c r="N7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>5005</v>
       </c>
@@ -908,19 +1040,23 @@
         <v>1</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="L8">
-        <v>5</v>
-      </c>
-      <c r="M8" t="s">
+        <v>800</v>
+      </c>
+      <c r="M8">
+        <v>1500</v>
+      </c>
+      <c r="N8" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>5006</v>
       </c>
@@ -949,19 +1085,23 @@
         <v>1</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K9">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="L9">
-        <v>5</v>
-      </c>
-      <c r="M9" t="s">
+        <v>800</v>
+      </c>
+      <c r="M9">
+        <v>1500</v>
+      </c>
+      <c r="N9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>5007</v>
       </c>
@@ -990,19 +1130,23 @@
         <v>1</v>
       </c>
       <c r="J10">
-        <v>5</v>
+        <v>800</v>
       </c>
       <c r="K10">
-        <v>3</v>
+        <f>J10-100</f>
+        <v>700</v>
       </c>
       <c r="L10">
-        <v>5</v>
-      </c>
-      <c r="M10" t="s">
+        <v>800</v>
+      </c>
+      <c r="M10">
+        <v>1500</v>
+      </c>
+      <c r="N10" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>5008</v>
       </c>
@@ -1031,15 +1175,19 @@
         <v>1</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K11">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="L11">
-        <v>5</v>
-      </c>
-      <c r="M11" t="s">
+        <v>800</v>
+      </c>
+      <c r="M11">
+        <v>1500</v>
+      </c>
+      <c r="N11" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1047,5 +1195,6 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🚧 wip: Monster AI Chasing/Attacking 80% 작업 완료
🐛 bugfix
- 이동시 몬스터가 이동하는 방향으로 몸체가 회전하지 않는 문제 해결

- 클라이언트와 서버의 몬스터 이동 속도 불일치로 인한 동기화 오류 해결

- 클라이언트에서 몬스터가 의도하지 않은 방향으로 이동하는 문제 해결
</commit_message>
<xml_diff>
--- a/Server/Common/GameDatasheet/Original_Monster.xlsx
+++ b/Server/Common/GameDatasheet/Original_Monster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zmwps\Desktop\Project_MMORPG\Server\Common\GameDatasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45BC756-4F2C-420E-BFFD-E48E38C4BB5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE30AABD-C3BF-4248-837F-1780C7E3BAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{1E70E408-E624-4B81-99D5-889082593FF6}"/>
   </bookViews>
@@ -24,80 +24,6 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>윤형석</author>
-  </authors>
-  <commentList>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{C371950D-C514-4F32-9E11-F3BC3AC117EC}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="돋움"/>
-            <family val="3"/>
-            <charset val="129"/>
-          </rPr>
-          <t>윤형석</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="돋움"/>
-            <family val="3"/>
-            <charset val="129"/>
-          </rPr>
-          <t>공격</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="돋움"/>
-            <family val="3"/>
-            <charset val="129"/>
-          </rPr>
-          <t>사거리</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
   <si>
@@ -120,18 +46,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>attack_range</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>detection_range</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>chase_range</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>gold_reward</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -299,7 +217,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>attack_attack_range</t>
+    <t>try_attack_range</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>is_targeting</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chasing_max_range</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -307,7 +233,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -322,34 +248,6 @@
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="돋움"/>
-      <family val="3"/>
-      <charset val="129"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="돋움"/>
-      <family val="3"/>
-      <charset val="129"/>
     </font>
   </fonts>
   <fills count="2">
@@ -691,7 +589,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{424A49E2-B413-473B-95D1-65DE3060862F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{424A49E2-B413-473B-95D1-65DE3060862F}">
   <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
@@ -700,7 +598,7 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -709,81 +607,81 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
-        <v>9</v>
-      </c>
       <c r="H1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
+        <v>52</v>
+      </c>
+      <c r="L1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>54</v>
       </c>
-      <c r="L1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M1" t="s">
-        <v>7</v>
-      </c>
       <c r="N1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.4">
@@ -794,32 +692,31 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>50</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>10</v>
       </c>
-      <c r="G3" t="s">
-        <v>39</v>
-      </c>
       <c r="H3" t="s">
-        <v>30</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
+        <v>37</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
       </c>
       <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
         <v>100</v>
-      </c>
-      <c r="K3">
-        <f>J3-50</f>
-        <v>50</v>
       </c>
       <c r="L3">
         <v>800</v>
@@ -828,7 +725,7 @@
         <v>1500</v>
       </c>
       <c r="N3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.4">
@@ -839,32 +736,31 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4">
+        <v>10</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4">
         <v>120</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>20</v>
       </c>
-      <c r="G4" t="s">
-        <v>22</v>
-      </c>
       <c r="H4" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>29</v>
       </c>
       <c r="J4">
-        <v>800</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <f>J4-100</f>
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="L4">
         <v>800</v>
@@ -873,7 +769,7 @@
         <v>1500</v>
       </c>
       <c r="N4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.4">
@@ -884,32 +780,31 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>200</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>40</v>
       </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
       <c r="H5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
+        <v>21</v>
+      </c>
+      <c r="I5" t="s">
+        <v>30</v>
       </c>
       <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
         <v>100</v>
-      </c>
-      <c r="K5">
-        <f t="shared" ref="K4:K11" si="0">J5-50</f>
-        <v>50</v>
       </c>
       <c r="L5">
         <v>800</v>
@@ -918,7 +813,7 @@
         <v>1500</v>
       </c>
       <c r="N5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.4">
@@ -929,32 +824,31 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6">
         <v>350</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>60</v>
       </c>
-      <c r="G6" t="s">
-        <v>24</v>
-      </c>
       <c r="H6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
+        <v>22</v>
+      </c>
+      <c r="I6" t="s">
+        <v>31</v>
       </c>
       <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
         <v>100</v>
-      </c>
-      <c r="K6">
-        <f t="shared" si="0"/>
-        <v>50</v>
       </c>
       <c r="L6">
         <v>800</v>
@@ -963,7 +857,7 @@
         <v>1500</v>
       </c>
       <c r="N6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.4">
@@ -974,32 +868,31 @@
         <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7">
+        <v>10</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7">
         <v>600</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>80</v>
       </c>
-      <c r="G7" t="s">
-        <v>25</v>
-      </c>
       <c r="H7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
+        <v>23</v>
+      </c>
+      <c r="I7" t="s">
+        <v>32</v>
       </c>
       <c r="J7">
-        <v>800</v>
+        <v>1</v>
       </c>
       <c r="K7">
-        <f>J7-100</f>
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="L7">
         <v>800</v>
@@ -1008,7 +901,7 @@
         <v>1500</v>
       </c>
       <c r="N7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.4">
@@ -1019,32 +912,31 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8">
+        <v>9</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8">
         <v>1000</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>120</v>
       </c>
-      <c r="G8" t="s">
-        <v>26</v>
-      </c>
       <c r="H8" t="s">
-        <v>35</v>
-      </c>
-      <c r="I8">
-        <v>1</v>
+        <v>24</v>
+      </c>
+      <c r="I8" t="s">
+        <v>33</v>
       </c>
       <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
         <v>100</v>
-      </c>
-      <c r="K8">
-        <f t="shared" si="0"/>
-        <v>50</v>
       </c>
       <c r="L8">
         <v>800</v>
@@ -1053,7 +945,7 @@
         <v>1500</v>
       </c>
       <c r="N8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.4">
@@ -1064,32 +956,31 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9">
+        <v>9</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9">
         <v>1500</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>180</v>
       </c>
-      <c r="G9" t="s">
-        <v>27</v>
-      </c>
       <c r="H9" t="s">
-        <v>36</v>
-      </c>
-      <c r="I9">
-        <v>1</v>
+        <v>25</v>
+      </c>
+      <c r="I9" t="s">
+        <v>34</v>
       </c>
       <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
         <v>100</v>
-      </c>
-      <c r="K9">
-        <f t="shared" si="0"/>
-        <v>50</v>
       </c>
       <c r="L9">
         <v>800</v>
@@ -1098,7 +989,7 @@
         <v>1500</v>
       </c>
       <c r="N9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.4">
@@ -1109,32 +1000,31 @@
         <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10">
+        <v>10</v>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10">
         <v>2000</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>240</v>
       </c>
-      <c r="G10" t="s">
-        <v>28</v>
-      </c>
       <c r="H10" t="s">
-        <v>37</v>
-      </c>
-      <c r="I10">
-        <v>1</v>
+        <v>26</v>
+      </c>
+      <c r="I10" t="s">
+        <v>35</v>
       </c>
       <c r="J10">
-        <v>800</v>
+        <v>1</v>
       </c>
       <c r="K10">
-        <f>J10-100</f>
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="L10">
         <v>800</v>
@@ -1143,7 +1033,7 @@
         <v>1500</v>
       </c>
       <c r="N10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.4">
@@ -1154,32 +1044,31 @@
         <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11">
+        <v>9</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11">
         <v>3000</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>300</v>
       </c>
-      <c r="G11" t="s">
-        <v>29</v>
-      </c>
       <c r="H11" t="s">
-        <v>38</v>
-      </c>
-      <c r="I11">
-        <v>1</v>
+        <v>27</v>
+      </c>
+      <c r="I11" t="s">
+        <v>36</v>
       </c>
       <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11">
         <v>100</v>
-      </c>
-      <c r="K11">
-        <f t="shared" si="0"/>
-        <v>50</v>
       </c>
       <c r="L11">
         <v>800</v>
@@ -1188,13 +1077,12 @@
         <v>1500</v>
       </c>
       <c r="N11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
✅ done: Monster AI 완료
</commit_message>
<xml_diff>
--- a/Server/Common/GameDatasheet/Original_Monster.xlsx
+++ b/Server/Common/GameDatasheet/Original_Monster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zmwps\Desktop\Project_MMORPG\Server\Common\GameDatasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3942FD46-69D5-4D4E-B0A1-1B36980C0F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D80A76B-6342-4914-887D-83436887A215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="1872" windowWidth="24828" windowHeight="12204" xr2:uid="{1E70E408-E624-4B81-99D5-889082593FF6}"/>
   </bookViews>
@@ -729,7 +729,7 @@
         <v>300</v>
       </c>
       <c r="L3">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="M3">
         <v>900</v>
@@ -823,7 +823,7 @@
         <v>300</v>
       </c>
       <c r="L5">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="M5">
         <v>900</v>
@@ -870,7 +870,7 @@
         <v>300</v>
       </c>
       <c r="L6">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="M6">
         <v>900</v>
@@ -964,7 +964,7 @@
         <v>300</v>
       </c>
       <c r="L8">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="M8">
         <v>900</v>
@@ -1011,7 +1011,7 @@
         <v>300</v>
       </c>
       <c r="L9">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="M9">
         <v>900</v>
@@ -1105,7 +1105,7 @@
         <v>300</v>
       </c>
       <c r="L11">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="M11">
         <v>900</v>

</xml_diff>